<commit_message>
Show unit-rate precision in takeoff workbook
</commit_message>
<xml_diff>
--- a/public/samples/spreadsheets/polypdf-construction-takeoff-template.xlsx
+++ b/public/samples/spreadsheets/polypdf-construction-takeoff-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimate" sheetId="1" r:id="Ra73b2b1fbadc48ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSV example" sheetId="2" r:id="Rc8c006f566674d9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimate" sheetId="1" r:id="R52161f376c1d4f64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSV example" sheetId="2" r:id="Rd32bcde35f2146e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,11 +14,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="&quot;$&quot;#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
-    <x:numFmt numFmtId="202" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0.00##"/>
     <x:numFmt numFmtId="203" formatCode="0.0%"/>
+    <x:numFmt numFmtId="204" formatCode="&quot;$&quot;#,##0.00##"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -152,7 +153,7 @@
     <x:xf numFmtId="202" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="204" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">

</xml_diff>